<commit_message>
Corrige asociaciones del acta y EPIG y equilibra logotipos
</commit_message>
<xml_diff>
--- a/documentos/01.2 Gestion Plan.xlsx
+++ b/documentos/01.2 Gestion Plan.xlsx
@@ -2367,7 +2367,7 @@
       </c>
       <c r="N2" s="19" t="inlineStr">
         <is>
-          <t>2.1; 2.2; 2.3; 2.4; 21; audio «Reunión Leyre julio» (15/07/2026); 27 (informe IKEI v1, PDF, e informe de cotejo del III Plan con REGCON, DOCX); 28 (informe IKEI v2, PDF, y análisis de pertinencia de las recomendaciones, DOCX). Los números 27 y 28 agrupan cuatro documentos.</t>
+          <t>2; 2.1; 2.2; 2.3; 2.4; 21; audio «Reunión Leyre julio» (15/07/2026); 27 (informe IKEI v1, PDF, e informe de cotejo del III Plan con REGCON, DOCX); 28 (informe IKEI v2, PDF, y análisis de pertinencia de las recomendaciones, DOCX). Los números 27 y 28 agrupan cuatro documentos.</t>
         </is>
       </c>
       <c r="O2" s="4" t="inlineStr">
@@ -3104,8 +3104,10 @@
 Como aportación adicional, la EIG incluyó un análisis exhaustivo del uso del lenguaje no sexista en las bases, identificando 46 expresiones que requerían corrección (26 desdoblamientos con barra inadecuados para texto normativo, 1 uso de arroba, 10 masculinos genéricos y 9 expresiones mejorables) y proponiendo reformulaciones siguiendo las directrices de Emakunde. Las correcciones fueron aceptadas e incorporadas antes de la publicación definitiva.</t>
         </is>
       </c>
-      <c r="N11" s="4" t="n">
-        <v>8</v>
+      <c r="N11" s="4" t="inlineStr">
+        <is>
+          <t>8; 23; 24</t>
+        </is>
       </c>
       <c r="O11" s="4" t="inlineStr">
         <is>

</xml_diff>